<commit_message>
Superatoms big set: +0 drawings, 250 API reads, 0 CXMolScribe reads
C-MAGE big superatoms: +0 drawings ({}), 250 read by Sonnet 5.5 API ($7.55), 0 by CXMolScribe; 600 read in all, PROTACs 201/2000; big-set API $19.54/140.
Exact: USPTO: API 63/100 63.0%, CX 54/100 54.0%; USPTO-ODP: API 368/500 73.6%, CX 298/500 59.6%

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/benchmarks/published_runs/sonnet55_api_superatoms/cxmolscribe/Completed_LowConfidence_CMAGE.xlsx
+++ b/benchmarks/published_runs/sonnet55_api_superatoms/cxmolscribe/Completed_LowConfidence_CMAGE.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K892"/>
+  <dimension ref="A1:K968"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26319,6 +26319,2210 @@
       </c>
       <c r="K892" t="inlineStr"/>
     </row>
+    <row r="893">
+      <c r="A893" s="1" t="n">
+        <v>891</v>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0362.png</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr"/>
+      <c r="D893" t="inlineStr"/>
+      <c r="E893" t="inlineStr"/>
+      <c r="F893" t="inlineStr">
+        <is>
+          <t>[H]C1(C(=O)NC(C(=O)N2CC(O)CC2C(=O)NC(CC(=O)NCCOCCOCCOCCNC(=O)CN2CCN(C(=O)C3=CC(F)=C(NC4=NC(C5CC5)=CN56C7C89=CNN=C8C78(=CNN=C8)C95=CN5=C46N=C5)C=C3)CC2)C2=CC=C(C3=C(C)N=CS3)C=C2)C(C)(C)C)CC1</t>
+        </is>
+      </c>
+      <c r="G893" t="inlineStr"/>
+      <c r="H893" t="inlineStr"/>
+      <c r="I893" t="n">
+        <v>0.1252789507773663</v>
+      </c>
+      <c r="J893" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K893" t="inlineStr"/>
+    </row>
+    <row r="894">
+      <c r="A894" s="1" t="n">
+        <v>892</v>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0364.png</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr"/>
+      <c r="D894" t="inlineStr"/>
+      <c r="E894" t="inlineStr"/>
+      <c r="F894" t="inlineStr">
+        <is>
+          <t>CCn1nc(C)cc1C(=O)Nc1nc2cc(C(N)=O)cc3c2n1C/C=C/Cn1c(NC(=O)c2cc(C)nn2CC)nc2cc(C(N)=O)cc(c21)OCC(N1CC2CCC(C1)O2)CO3</t>
+        </is>
+      </c>
+      <c r="G894" t="inlineStr"/>
+      <c r="H894" t="inlineStr"/>
+      <c r="I894" t="n">
+        <v>0.8167903231438567</v>
+      </c>
+      <c r="J894" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K894" t="inlineStr"/>
+    </row>
+    <row r="895">
+      <c r="A895" s="1" t="n">
+        <v>893</v>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0366.png</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr"/>
+      <c r="D895" t="inlineStr"/>
+      <c r="E895" t="inlineStr"/>
+      <c r="F895" t="inlineStr">
+        <is>
+          <t>CC(C)(C)C(=O)OCOP1(=O)OCOC2(=O)C(C)(C)(C)C(=O)(OCOP3(=O)(OCOC(=O)C(C)(C)C)CO3CC3OC(N4C=NC5=C4N=CN=C5N)C(F)C3OP3(=O)OC[CH]45C(O3)[CH]36OCC7N89C=NC%10%11=C8N=CN=C%10(N)=N8=C%11(N)C%10=C(N=C8)N(C=N%10)[CH]9(CO43)[CH]756O1)C2(C)(C)C</t>
+        </is>
+      </c>
+      <c r="G895" t="inlineStr"/>
+      <c r="H895" t="inlineStr"/>
+      <c r="I895" t="n">
+        <v>0.001817076448464142</v>
+      </c>
+      <c r="J895" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K895" t="inlineStr"/>
+    </row>
+    <row r="896">
+      <c r="A896" s="1" t="n">
+        <v>894</v>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0367.png</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr"/>
+      <c r="D896" t="inlineStr"/>
+      <c r="E896" t="inlineStr"/>
+      <c r="F896" t="inlineStr">
+        <is>
+          <t>CC1=NOC(C(C(=O)N2CC(O)CC2C(=O)NC(CC(=O)NCCCCCCCNC(=O)CN2CCN(C(=O)C3=CC(F)=C(NC45=NC(C6CC6)=C6N789C%10%11%12=C%13=C7%14%15(=C7N%16=C48%17=N7%13=C=%1659N6%10%17%14)C%114=C5=C%12%1567=C8NN9=C6=N(=C=947)N85)C=C3)CC2)C2=CC=C(C3=C(C)N=CS3)C=C2)C(C)(C)C)=C1</t>
+        </is>
+      </c>
+      <c r="G896" t="inlineStr"/>
+      <c r="H896" t="inlineStr"/>
+      <c r="I896" t="n">
+        <v>0.01698433611194213</v>
+      </c>
+      <c r="J896" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K896" t="inlineStr"/>
+    </row>
+    <row r="897">
+      <c r="A897" s="1" t="n">
+        <v>895</v>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0379.png</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr"/>
+      <c r="D897" t="inlineStr"/>
+      <c r="E897" t="inlineStr"/>
+      <c r="F897" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC1=NC23=C4C(=CC(C(N)=O)=C2)OCC(N2CCC(C#N)CC2)COC2=CC(C(N)=O)=CC56=C27N(CC=CCN1)C(NC(=O)C1=CC(C)=NN1CC)(=N5)N7(CC=CCN4C(NC(=O)C1=CC(C)=NN1CC)=N3)C(NC(=O)C1=CC(C)=NN1CC)=N6</t>
+        </is>
+      </c>
+      <c r="G897" t="inlineStr"/>
+      <c r="H897" t="inlineStr"/>
+      <c r="I897" t="n">
+        <v>0.3970236958179507</v>
+      </c>
+      <c r="J897" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K897" t="inlineStr"/>
+    </row>
+    <row r="898">
+      <c r="A898" s="1" t="n">
+        <v>896</v>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0386.png</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr"/>
+      <c r="D898" t="inlineStr"/>
+      <c r="E898" t="inlineStr"/>
+      <c r="F898" t="inlineStr">
+        <is>
+          <t>Cn1cc(-c2cccc(C(F)(F)F)c2)c2sc(C(=O)NC3CC4(CCN(c5ccc6c(c5)C(=O)N(C5CCC(=O)NC5=O)C6)CC4)C3)cc2c1=O</t>
+        </is>
+      </c>
+      <c r="G898" t="inlineStr"/>
+      <c r="H898" t="inlineStr"/>
+      <c r="I898" t="n">
+        <v>0.8178532882779922</v>
+      </c>
+      <c r="J898" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K898" t="inlineStr"/>
+    </row>
+    <row r="899">
+      <c r="A899" s="1" t="n">
+        <v>897</v>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0388.png</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr"/>
+      <c r="D899" t="inlineStr"/>
+      <c r="E899" t="inlineStr"/>
+      <c r="F899" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC12=NC3=C45C(=CC(C(N)=O)=C3)OCC(N3CCC(OP(=O)(OC(C)(C)C)OC(C)(C)C)C3)COC3=CC(C(N)=O)=CC67=C38N39CC=CCN14CC=CCN81C348%10=N6=C913(=N=47)N(CC=CCN25)CNC(=O)C1=CC(C)=NN1(CC)C1(=CC2=NN1(CC)C1(=CC(C)(=NN1CC)C2)C(=O)N8)C(=O)N%103</t>
+        </is>
+      </c>
+      <c r="G899" t="inlineStr"/>
+      <c r="H899" t="inlineStr"/>
+      <c r="I899" t="n">
+        <v>0.01271708829738312</v>
+      </c>
+      <c r="J899" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K899" t="inlineStr"/>
+    </row>
+    <row r="900">
+      <c r="A900" s="1" t="n">
+        <v>898</v>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0399.png</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr"/>
+      <c r="D900" t="inlineStr"/>
+      <c r="E900" t="inlineStr"/>
+      <c r="F900" t="inlineStr">
+        <is>
+          <t>CC(C)C(NC(=O)CCOCCOCCOCCC(=O)NCCN1CCN(C(=O)C2=CC(F)=C(NC34=NC(C5CC5)=C5N678C9%10=C%11=C6%12%13(=CN6=C37N59%12C=648=N%11)C3(=CNN=C3)C3=NNC=C3%10%13)C=C2)CC1)C(=O)N1CC(O)CC1C(=O)NCC1=CC=C(C2=CN=CS2)C=C1</t>
+        </is>
+      </c>
+      <c r="G900" t="inlineStr"/>
+      <c r="H900" t="inlineStr"/>
+      <c r="I900" t="n">
+        <v>0.03670332202610745</v>
+      </c>
+      <c r="J900" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K900" t="inlineStr"/>
+    </row>
+    <row r="901">
+      <c r="A901" s="1" t="n">
+        <v>899</v>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0402.png</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr"/>
+      <c r="D901" t="inlineStr"/>
+      <c r="E901" t="inlineStr"/>
+      <c r="F901" t="inlineStr">
+        <is>
+          <t>CCC(C)(C)C(=O)OCOP12(=O)OCOC(=O)C(C)(C)(CC)C(=O)(C(C)(C)CC)OCCOCC3O[CH]456C(F)[CH]3789%10OP3(=O)OC[CH]C(O1)O2P1(=O)(OCOC(=O)C(C)(C)CC)C2C1O2C[CH]71O4C([CH]8(F)[CH]19O3%10)N51C=NC2=C1N=CN=C2(N)C12=C(N=CN=C1N)N6C=N2</t>
+        </is>
+      </c>
+      <c r="G901" t="inlineStr"/>
+      <c r="H901" t="inlineStr"/>
+      <c r="I901" t="n">
+        <v>0.01257274257374918</v>
+      </c>
+      <c r="J901" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K901" t="inlineStr"/>
+    </row>
+    <row r="902">
+      <c r="A902" s="1" t="n">
+        <v>900</v>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0403.png</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr"/>
+      <c r="D902" t="inlineStr"/>
+      <c r="E902" t="inlineStr"/>
+      <c r="F902" t="inlineStr">
+        <is>
+          <t>CC1=C(C2=CC=C(C(CC(=O)NCCCCCNC(=O)CN3CCN(C(=O)C4=CC(F)=C(NC56=NC(C7CC7)=C7N89%10C%11%12%13=C%14=C8%15%16(=C8N%14=C59%14%17=N8=C6%10%14N7%11%15%17)C%125=C6=C%13%1678=C9NN%10=C7=N(=C=%1058)N96)C=C4)CC3)NC(=O)C3CC(O)CN3C(=O)C(NC(=O)C3(F)CC3)C(C)(C)C)C=C2)SC=N1</t>
+        </is>
+      </c>
+      <c r="G902" t="inlineStr"/>
+      <c r="H902" t="inlineStr"/>
+      <c r="I902" t="n">
+        <v>0.01105399300597473</v>
+      </c>
+      <c r="J902" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K902" t="inlineStr"/>
+    </row>
+    <row r="903">
+      <c r="A903" s="1" t="n">
+        <v>901</v>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0405.png</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr"/>
+      <c r="D903" t="inlineStr"/>
+      <c r="E903" t="inlineStr"/>
+      <c r="F903" t="inlineStr">
+        <is>
+          <t>Cc1ncsc1-c1ccc(CNC(=O)[C@@H]2C[C@@H](O)CN2C(=O)[C@@H](NC(=O)COCC(=O)NCCN2CCN(C(=O)c3ccc(Nc4nc(C5CC5)cn5c(-c6cn[nH]c6)cnc45)c(F)c3)CC2)C(C)(C)C)cc1</t>
+        </is>
+      </c>
+      <c r="G903" t="inlineStr"/>
+      <c r="H903" t="inlineStr"/>
+      <c r="I903" t="n">
+        <v>0.8232431779310004</v>
+      </c>
+      <c r="J903" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K903" t="inlineStr"/>
+    </row>
+    <row r="904">
+      <c r="A904" s="1" t="n">
+        <v>902</v>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0408.png</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr"/>
+      <c r="D904" t="inlineStr"/>
+      <c r="E904" t="inlineStr"/>
+      <c r="F904" t="inlineStr">
+        <is>
+          <t>Cc1cc(-c2nc(-c3ccc(N4CCC(CN5CCC6(CC5)COc5cc7c(cc56)C(=O)N(C5CCC(=O)NC5=O)C7=O)CC4)nc3)cn3nccc23)ccc1[C@@H](C)NC(=O)c1nnn(C(C)(C)C)n1</t>
+        </is>
+      </c>
+      <c r="G904" t="inlineStr"/>
+      <c r="H904" t="inlineStr"/>
+      <c r="I904" t="n">
+        <v>0.7983359986010865</v>
+      </c>
+      <c r="J904" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K904" t="inlineStr"/>
+    </row>
+    <row r="905">
+      <c r="A905" s="1" t="n">
+        <v>903</v>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0416.png</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr"/>
+      <c r="D905" t="inlineStr"/>
+      <c r="E905" t="inlineStr"/>
+      <c r="F905" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC1=NC2=C3N1CC=CCN145C6=C7C8=C(C(N)=O)C=C69OCC(N6CCC(O)C6)N6(CCC(O)C6)C6%10COC3(=CC(C(N)=O)=C2)OCC(N2CCC(O)C2)C6O2CC913=C81(C=C(C(N)=O)C=C23OC%10)N=C42(NC(=O)C3=CC(C)=NN3CC)=N71=C25NC(=O)C1=CC(C)=NN1CC</t>
+        </is>
+      </c>
+      <c r="G905" t="inlineStr"/>
+      <c r="H905" t="inlineStr"/>
+      <c r="I905" t="n">
+        <v>0.004514561475377862</v>
+      </c>
+      <c r="J905" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K905" t="inlineStr"/>
+    </row>
+    <row r="906">
+      <c r="A906" s="1" t="n">
+        <v>904</v>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0417.png</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr"/>
+      <c r="D906" t="inlineStr"/>
+      <c r="E906" t="inlineStr"/>
+      <c r="F906" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC1=NC2=C3C(=CC(C(N)=O)=C2)OCC(N2CCC(OP(=O)(O)O)C2)COC24=CC(C(N)=O)=CC567=C2(C=C=4C(C(N)=O)=C5)N(CC=CCN13)(C(NC(=O)C1=CC(C)=NN1CC)=N6)C(NC(=O)C1=CC(C)=NN1CC)=N7.S</t>
+        </is>
+      </c>
+      <c r="G906" t="inlineStr"/>
+      <c r="H906" t="inlineStr"/>
+      <c r="I906" t="n">
+        <v>0.5106671102894167</v>
+      </c>
+      <c r="J906" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K906" t="inlineStr"/>
+    </row>
+    <row r="907">
+      <c r="A907" s="1" t="n">
+        <v>905</v>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0422.png</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr"/>
+      <c r="D907" t="inlineStr"/>
+      <c r="E907" t="inlineStr"/>
+      <c r="F907" t="inlineStr">
+        <is>
+          <t>[H]C12CC(C)(C)C(C(=O)NC3C4=CC=CCC4=CC3OCC#CC#CCO[CH]3=CC4=C(C=CC=C4)C3NC(=O)C3N4C(=O)C(NC(=O)C(C)NC)CCOC4([H])CC3(C)C)N1C(=O)C(NC(=O)C(C)NC)CCO2</t>
+        </is>
+      </c>
+      <c r="G907" t="inlineStr"/>
+      <c r="H907" t="inlineStr"/>
+      <c r="I907" t="n">
+        <v>0.5820154437331464</v>
+      </c>
+      <c r="J907" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K907" t="inlineStr"/>
+    </row>
+    <row r="908">
+      <c r="A908" s="1" t="n">
+        <v>906</v>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0423.png</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr"/>
+      <c r="D908" t="inlineStr"/>
+      <c r="E908" t="inlineStr"/>
+      <c r="F908" t="inlineStr">
+        <is>
+          <t>COC(=O)c1cccc(CN2CCOCCOCCN(Cc3cc(OCCc4ccc(NC(=O)OC(C)(C)C)cc4)cc(C(=O)OC)n3)CCOCCOCC2)n1</t>
+        </is>
+      </c>
+      <c r="G908" t="inlineStr"/>
+      <c r="H908" t="inlineStr"/>
+      <c r="I908" t="n">
+        <v>0.7498794691086894</v>
+      </c>
+      <c r="J908" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K908" t="inlineStr"/>
+    </row>
+    <row r="909">
+      <c r="A909" s="1" t="n">
+        <v>907</v>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0428.png</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr"/>
+      <c r="D909" t="inlineStr"/>
+      <c r="E909" t="inlineStr"/>
+      <c r="F909" t="inlineStr">
+        <is>
+          <t>CC(C)(C)Cc1cc(CSC[C@H](N)C(=O)O)cc(CN2CCN(C(=O)CN3CCN(CC(=O)O)CCN(CC(=O)O)CCN(CC(=O)O)CC3)CC2)c1</t>
+        </is>
+      </c>
+      <c r="G909" t="inlineStr"/>
+      <c r="H909" t="inlineStr"/>
+      <c r="I909" t="n">
+        <v>0.6288647608549713</v>
+      </c>
+      <c r="J909" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K909" t="inlineStr"/>
+    </row>
+    <row r="910">
+      <c r="A910" s="1" t="n">
+        <v>908</v>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0436.png</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr"/>
+      <c r="D910" t="inlineStr"/>
+      <c r="E910" t="inlineStr"/>
+      <c r="F910" t="inlineStr">
+        <is>
+          <t>CCn1c(-c2cc(N3CCN4CCOCC4C3)cnc2C(C)OC)c2c3cc(ccc31)-c1csc(n1)CC(NC(=O)C1C(C)C1C)C(=O)N1NC(C(=O)OCC(C)(C)C2)C2CC1C2</t>
+        </is>
+      </c>
+      <c r="G910" t="inlineStr"/>
+      <c r="H910" t="inlineStr"/>
+      <c r="I910" t="n">
+        <v>0.7090422626759315</v>
+      </c>
+      <c r="J910" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K910" t="inlineStr"/>
+    </row>
+    <row r="911">
+      <c r="A911" s="1" t="n">
+        <v>909</v>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0439.png</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr"/>
+      <c r="D911" t="inlineStr"/>
+      <c r="E911" t="inlineStr"/>
+      <c r="F911" t="inlineStr">
+        <is>
+          <t>CC(C)NC(=O)C1CC(O)CN1C(=O)C(NC(=O)COCCOCCOCCNC(=O)CN12CCN3C4(=O)N(CC1)(CC2)C31(=O)C2=C3=C4156=CC(F)=C14C=C5=C157=C=62=CC5(=C3F)NC123=C56=C89%10%11=C%12%13C5%14=C=85%15N%128%16%17C%12%18%19=C%20=C8%21%22%23(C8=CNN=C8)=CN=C1%168%24%25C=71%16=N7=C%26C21%27%28=N1=C%263%16%17(=N%20)(C6%278(=N9)N4)(N%13%125%24%21)N%18%15%28%25%22(C=C7C2CC2C%14%102CC2C%112CC2)C2(=C1)C1=CN3N=C1C2%19%231=C3NN=C1)C(C)C</t>
+        </is>
+      </c>
+      <c r="G911" t="inlineStr"/>
+      <c r="H911" t="inlineStr"/>
+      <c r="I911" t="n">
+        <v>4.983511845494615e-07</v>
+      </c>
+      <c r="J911" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K911" t="inlineStr"/>
+    </row>
+    <row r="912">
+      <c r="A912" s="1" t="n">
+        <v>910</v>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0449.png</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr"/>
+      <c r="D912" t="inlineStr"/>
+      <c r="E912" t="inlineStr"/>
+      <c r="F912" t="inlineStr">
+        <is>
+          <t>[H]C12CC(C)(C)C(C(=O)NC3C4=C(C=CC=C4)CC3OCC3=CC=C(C#CCO[CH]4=CC5=C(C=CC=C5)C4NC(=O)C4N5C(=O)C(NC(=O)C(C)N(C)C(=O)OC(C)(C)C)CCSC5([H])CC4(C)C)C=C3)N1C(=O)C(NC(=O)C(C)N(C)C(=O)OC(C)(C)C)CCS2</t>
+        </is>
+      </c>
+      <c r="G912" t="inlineStr"/>
+      <c r="H912" t="inlineStr"/>
+      <c r="I912" t="n">
+        <v>0.5264108564159679</v>
+      </c>
+      <c r="J912" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K912" t="inlineStr"/>
+    </row>
+    <row r="913">
+      <c r="A913" s="1" t="n">
+        <v>911</v>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0452.png</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr"/>
+      <c r="D913" t="inlineStr"/>
+      <c r="E913" t="inlineStr"/>
+      <c r="F913" t="inlineStr">
+        <is>
+          <t>CC1=C(C2=CC=C(CNC(=O)C3CC(O)CN3C(=O)C(NC(=O)C3(F)CC3)C(C)(C)C)C(OCCCCNC(=O)CN3CCN(C(=O)C4=CC(F)=C(NC5N=C(C6CC6)C=N6C(C7=CNN=C7)=CN=C56)C=C4)CC3)=C2)SC=N1</t>
+        </is>
+      </c>
+      <c r="G913" t="inlineStr"/>
+      <c r="H913" t="inlineStr"/>
+      <c r="I913" t="n">
+        <v>0.7613854620640638</v>
+      </c>
+      <c r="J913" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K913" t="inlineStr"/>
+    </row>
+    <row r="914">
+      <c r="A914" s="1" t="n">
+        <v>912</v>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0456.png</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr"/>
+      <c r="D914" t="inlineStr"/>
+      <c r="E914" t="inlineStr"/>
+      <c r="F914" t="inlineStr">
+        <is>
+          <t>O=C(O)CCC(NC(=O)NC(CCCCN(Cc1ccc(Br)cc1)C(=O)CCCCCNC(=O)CN1CCN(CC(=O)O)CCN(CC(=O)O)CCN(CC(=O)O)CC1)C(=O)O)C(=O)O</t>
+        </is>
+      </c>
+      <c r="G914" t="inlineStr"/>
+      <c r="H914" t="inlineStr"/>
+      <c r="I914" t="n">
+        <v>0.8137497071408518</v>
+      </c>
+      <c r="J914" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K914" t="inlineStr"/>
+    </row>
+    <row r="915">
+      <c r="A915" s="1" t="n">
+        <v>913</v>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0457.png</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr"/>
+      <c r="D915" t="inlineStr"/>
+      <c r="E915" t="inlineStr"/>
+      <c r="F915" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC=NC1=C23C4=CC(C(N)=O)=C1C1=C5N2CC=CCN26C7=CC8=C(C(N)=O)C=C7(OCC(N7CCC(O)CC7)CO4)C24=C8(C=C(C(N)=O)C=C4OCC(N2CCC(O)CC2)COC53=CC(C(N)=O)=C1)N=C6NC(=O)C1=CC(C)=NN1CC</t>
+        </is>
+      </c>
+      <c r="G915" t="inlineStr"/>
+      <c r="H915" t="inlineStr"/>
+      <c r="I915" t="n">
+        <v>0.1951681135951842</v>
+      </c>
+      <c r="J915" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K915" t="inlineStr"/>
+    </row>
+    <row r="916">
+      <c r="A916" s="1" t="n">
+        <v>914</v>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0458.png</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr"/>
+      <c r="D916" t="inlineStr"/>
+      <c r="E916" t="inlineStr"/>
+      <c r="F916" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC1=NC23=C4N1CC=CCN15C(NC(=O)C6=CC(C)=NN6CC)=NC67(=C18C1=C(=C8(=CC(C(N)=O)=C6)OCC68COC4(=CC(C(N)=O)=C2)O(C=CC(C(N)=O)=C3)CC(C6O1)N1CCC(C1)O([Si]1(C)(C)CC1(C)C)[CH]1(O[Si](C)(C)C(C)(C)C)CCN8C1)C(C(N)=O)=C7)N=C5NC(=O)C1=CC(C)=NN1CC</t>
+        </is>
+      </c>
+      <c r="G916" t="inlineStr"/>
+      <c r="H916" t="inlineStr"/>
+      <c r="I916" t="n">
+        <v>0.008252304500852051</v>
+      </c>
+      <c r="J916" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K916" t="inlineStr"/>
+    </row>
+    <row r="917">
+      <c r="A917" s="1" t="n">
+        <v>915</v>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0459.png</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr"/>
+      <c r="D917" t="inlineStr"/>
+      <c r="E917" t="inlineStr"/>
+      <c r="F917" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC1=NC2=C3N1CC=CCN145C6=C78C9=C(C(N)=O)C=C%10OCC(CCN%11CCOCC%11)COC3(=CC(C(N)=O)=C2)OCC(CCN2CCOCC2)COC62=CC(C(N)=O)=C7C93=C%1021NC41(NC(=O)C2=CC(C)=NN2CC)(=N3)=N8=C51NC(=O)C1=CC(C)=NN1CC</t>
+        </is>
+      </c>
+      <c r="G917" t="inlineStr"/>
+      <c r="H917" t="inlineStr"/>
+      <c r="I917" t="n">
+        <v>0.004148247425585713</v>
+      </c>
+      <c r="J917" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K917" t="inlineStr"/>
+    </row>
+    <row r="918">
+      <c r="A918" s="1" t="n">
+        <v>916</v>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0464.png</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr"/>
+      <c r="D918" t="inlineStr"/>
+      <c r="E918" t="inlineStr"/>
+      <c r="F918" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC=NC1=C23C4=CC(C(N)=O)=C1C1=C5N2CC=CCN26C7=CC8=C(C(N)=O)C=C7(OCC(C7CCNCC7)CO4)C24=C8(C=C(C(N)=O)C=C4OCC(C2CCNCC2)COC53=CC(C(N)=O)=C1)N=C6NC(=O)C1=CC(C)=NN1CC</t>
+        </is>
+      </c>
+      <c r="G918" t="inlineStr"/>
+      <c r="H918" t="inlineStr"/>
+      <c r="I918" t="n">
+        <v>0.1301031810989756</v>
+      </c>
+      <c r="J918" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K918" t="inlineStr"/>
+    </row>
+    <row r="919">
+      <c r="A919" s="1" t="n">
+        <v>917</v>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0465.png</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr"/>
+      <c r="D919" t="inlineStr"/>
+      <c r="E919" t="inlineStr"/>
+      <c r="F919" t="inlineStr">
+        <is>
+          <t>Cc1ncsc1-c1ccc(CNC(=O)[C@@H]2C[C@@H](O)CN2C(=O)[C@@H](NC(=O)CCCC(O)NCCCCn2cnc(-c3cnc(O[C@@H]4CCN(C(=O)Cc5ccc(OC(F)(F)F)cc5)C[C@H]4F)c(C(N)=O)c3)c2)C(C)(C)C)cc1</t>
+        </is>
+      </c>
+      <c r="G919" t="inlineStr"/>
+      <c r="H919" t="inlineStr"/>
+      <c r="I919" t="n">
+        <v>0.8430239027149971</v>
+      </c>
+      <c r="J919" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K919" t="inlineStr"/>
+    </row>
+    <row r="920">
+      <c r="A920" s="1" t="n">
+        <v>918</v>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0466.png</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr"/>
+      <c r="D920" t="inlineStr"/>
+      <c r="E920" t="inlineStr"/>
+      <c r="F920" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC1=NC2=C3C(=CC(C(N)=O)=C2)OCC(N2CCC(N)CC2)COC24=CC(C(N)=O)=CC567=C2(C(OCC(CO)N2CCC(N)CC2)=C=4C(C(N)=O)=C5)N2(CC=CCN13)C(NC(=O)C1=CC(C)=NN1CC)=N6C2(NC(=O)C1=CC(C)=NN1CC)=N7</t>
+        </is>
+      </c>
+      <c r="G920" t="inlineStr"/>
+      <c r="H920" t="inlineStr"/>
+      <c r="I920" t="n">
+        <v>0.1766539403401964</v>
+      </c>
+      <c r="J920" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K920" t="inlineStr"/>
+    </row>
+    <row r="921">
+      <c r="A921" s="1" t="n">
+        <v>919</v>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0470.png</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr"/>
+      <c r="D921" t="inlineStr"/>
+      <c r="E921" t="inlineStr"/>
+      <c r="F921" t="inlineStr">
+        <is>
+          <t>[H]C12CC(C)(C)C(C(=O)NC3C4=C(C=CC=C4)CC3OCC#CC3=CC=CC(C#CCO[CH]CC4=CC=CC=C4)=C3)N1C(=O)C(NC(=O)C(C)N(C)C(=O)OC(C)(C)C)CCS2.[H]C12CC3(C)(C)C4[CH]3(C(=O)NC3C5=C(C=CC=C5)CC3O)N41C(=O)C(NC(=O)C(C)N(C)C(=O)OC(C)(C)C)CCS2</t>
+        </is>
+      </c>
+      <c r="G921" t="inlineStr"/>
+      <c r="H921" t="inlineStr"/>
+      <c r="I921" t="n">
+        <v>0.2912964728985484</v>
+      </c>
+      <c r="J921" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K921" t="inlineStr"/>
+    </row>
+    <row r="922">
+      <c r="A922" s="1" t="n">
+        <v>920</v>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0471.png</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr"/>
+      <c r="D922" t="inlineStr"/>
+      <c r="E922" t="inlineStr"/>
+      <c r="F922" t="inlineStr">
+        <is>
+          <t>C=C1OC2C(CC3CCN(C)CC3)COC345=CC(C(N)=O)=CC6=C3N(CC=CCN378C9%10=C%11%12C%13=C(C(N)=O)C=C9%14OCC29%15(CO4)CC2(CCN(C)CC2)C9C(CO5)C%15OC%102=CC(C(N)=O)=C%11C%134(=C1%1423)N=C71(NC(=O)C2=CC(C)=NN2CC)=N%124=C18NC(=O)C1=CC(C)=NN1CC)C(NC(=O)C1=CC(C)=NN1CC)=N6</t>
+        </is>
+      </c>
+      <c r="G922" t="inlineStr"/>
+      <c r="H922" t="inlineStr"/>
+      <c r="I922" t="n">
+        <v>0.0008862207562917128</v>
+      </c>
+      <c r="J922" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K922" t="inlineStr"/>
+    </row>
+    <row r="923">
+      <c r="A923" s="1" t="n">
+        <v>921</v>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0473.png</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr"/>
+      <c r="D923" t="inlineStr"/>
+      <c r="E923" t="inlineStr"/>
+      <c r="F923" t="inlineStr">
+        <is>
+          <t>COC=C1CN2CC3CN4CCC56CC4N4(CCC789(CC4)CN(C7)C4=CC=C7%10(CN(C%11CCC(=O)NC%11=O)C(=O)C7=C4)C4C7=CC=C(C=C7%10C(=O)N4C4CCC(=O)NC4=O)N(C58)C69)CC4CN(CC5=C(OC)C=CC=C5(OC)C=C1OC)(C4)C32</t>
+        </is>
+      </c>
+      <c r="G923" t="inlineStr"/>
+      <c r="H923" t="inlineStr"/>
+      <c r="I923" t="n">
+        <v>0.01268095452392003</v>
+      </c>
+      <c r="J923" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K923" t="inlineStr"/>
+    </row>
+    <row r="924">
+      <c r="A924" s="1" t="n">
+        <v>922</v>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0476.png</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr"/>
+      <c r="D924" t="inlineStr"/>
+      <c r="E924" t="inlineStr"/>
+      <c r="F924" t="inlineStr">
+        <is>
+          <t>COP(=O)(S)O[CH]123O4[CH]56[CH]17(N1C=NC8=C1N=CN(CCNC(=O)CO)C8=O)O[CH]189%10COP(=O)(S)O[CH]%11(OP(=O)(S)OC1[CH]1(O78)[CH]529O[CH]163%10O)C(COP4(=O)S)OC(N1C=C2CCCSC3=NC=NC1=C23)C%11F</t>
+        </is>
+      </c>
+      <c r="G924" t="inlineStr"/>
+      <c r="H924" t="inlineStr"/>
+      <c r="I924" t="n">
+        <v>0.1059968933483516</v>
+      </c>
+      <c r="J924" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K924" t="inlineStr"/>
+    </row>
+    <row r="925">
+      <c r="A925" s="1" t="n">
+        <v>923</v>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0480.png</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr"/>
+      <c r="D925" t="inlineStr"/>
+      <c r="E925" t="inlineStr"/>
+      <c r="F925" t="inlineStr">
+        <is>
+          <t>[H]C12CC(C)(C)C(C(=O)NC3C4=CC=CCC4=CC3OCC#CC#CCO[CH]3=CC4=C(C=CC=C4)C3NC(=O)C3N4C(=O)C(NC(=O)C(CC)NC)CCSC4([H])CC3(C)C)N1C(=O)C(NC(=O)C(CC)NC)CCS2</t>
+        </is>
+      </c>
+      <c r="G925" t="inlineStr"/>
+      <c r="H925" t="inlineStr"/>
+      <c r="I925" t="n">
+        <v>0.5564464817718697</v>
+      </c>
+      <c r="J925" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K925" t="inlineStr"/>
+    </row>
+    <row r="926">
+      <c r="A926" s="1" t="n">
+        <v>924</v>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0487.png</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr"/>
+      <c r="D926" t="inlineStr"/>
+      <c r="E926" t="inlineStr"/>
+      <c r="F926" t="inlineStr">
+        <is>
+          <t>[H][C@]12CC(C)(C)[C@@H](C(=O)N[C@H]3c4ccccc4C[C@H]3OCCS(=O)(=O)CCO[C@@H]3Cc4ccccc4[C@@H]3NC(=O)[C@H]3N4C(=O)[C@@H](NC(=O)[C@H](C)N(C)C(=O)OC(C)(C)C)CCS[C@@]4(Cl)CC3(C)C)N1C(=O)[C@@H](NC(=O)[C@H](C)N(C)C(=O)OC(C)(C)C)CCS2</t>
+        </is>
+      </c>
+      <c r="G926" t="inlineStr"/>
+      <c r="H926" t="inlineStr"/>
+      <c r="I926" t="n">
+        <v>0.794726161022269</v>
+      </c>
+      <c r="J926" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K926" t="inlineStr"/>
+    </row>
+    <row r="927">
+      <c r="A927" s="1" t="n">
+        <v>925</v>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0494.png</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr"/>
+      <c r="D927" t="inlineStr"/>
+      <c r="E927" t="inlineStr"/>
+      <c r="F927" t="inlineStr">
+        <is>
+          <t>COC(=O)c1cc2c(c([N+](=O)[O-])c1)NC/C=C/CNc1c(cc(C(=O)OC)cc1[N+](=O)[O-])OCC(N1CC[C@H](O[Si](C)(C)C(C)(C)C)C1)CO2.S</t>
+        </is>
+      </c>
+      <c r="G927" t="inlineStr"/>
+      <c r="H927" t="inlineStr"/>
+      <c r="I927" t="n">
+        <v>0.7596514244874697</v>
+      </c>
+      <c r="J927" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K927" t="inlineStr"/>
+    </row>
+    <row r="928">
+      <c r="A928" s="1" t="n">
+        <v>926</v>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0496.png</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr"/>
+      <c r="D928" t="inlineStr"/>
+      <c r="E928" t="inlineStr"/>
+      <c r="F928" t="inlineStr">
+        <is>
+          <t>COC1=CC=CC(OC)=C1CN12CC3(CN45CCC678(CC4)CN(C6)C4=CC=C69%10C(=O)N(C%11CCC(=O)NC%11=O)(CC6=C4)C4C(C6CCC(=O)NC6=O)C9(=O)C6=CC=C(C=C64%10)N4C7C6(CCN(CC7CN(CC9=C(OC)C=C9)C731)C5C6)C48)C2</t>
+        </is>
+      </c>
+      <c r="G928" t="inlineStr"/>
+      <c r="H928" t="inlineStr"/>
+      <c r="I928" t="n">
+        <v>0.01062268003809441</v>
+      </c>
+      <c r="J928" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K928" t="inlineStr"/>
+    </row>
+    <row r="929">
+      <c r="A929" s="1" t="n">
+        <v>927</v>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0498.png</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr"/>
+      <c r="D929" t="inlineStr"/>
+      <c r="E929" t="inlineStr"/>
+      <c r="F929" t="inlineStr">
+        <is>
+          <t>CC1=C(C2=CC=C(CNC(=O)C3CC(O)CN3C(=O)C(NC(=O)CCOCCOCCOCCOCCNC(=O)CN3CCN(C(=O)C4=CC(F)=C(NC=NC(=CN5C678=CN=C569C756=CNN=C5C895=CNN=C65)C5CC5)C=C4)CC3)C(C)C)C=C2)SC=N1</t>
+        </is>
+      </c>
+      <c r="G929" t="inlineStr"/>
+      <c r="H929" t="inlineStr"/>
+      <c r="I929" t="n">
+        <v>0.2771900526634529</v>
+      </c>
+      <c r="J929" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K929" t="inlineStr"/>
+    </row>
+    <row r="930">
+      <c r="A930" s="1" t="n">
+        <v>928</v>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0500.png</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr"/>
+      <c r="D930" t="inlineStr"/>
+      <c r="E930" t="inlineStr"/>
+      <c r="F930" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC1=NC2=C3N1CC=CCN14C(NC(=O)C5=CC(C)=NN5CC)=NC56(=C17C1=C(=C7(=CC(C(N)=O)=C5)OCC5(N7CCC(OP(=O)(O)O)CC7)COC3(=CC(C(N)=O)=C2)OCC(N2CCC(OP(=O)(O)O)CC2)C5O1)C(C(N)=O)=C6)N=C4NC(=O)C1=CC(C)=NN1CC</t>
+        </is>
+      </c>
+      <c r="G930" t="inlineStr"/>
+      <c r="H930" t="inlineStr"/>
+      <c r="I930" t="n">
+        <v>0.1039793297318868</v>
+      </c>
+      <c r="J930" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K930" t="inlineStr"/>
+    </row>
+    <row r="931">
+      <c r="A931" s="1" t="n">
+        <v>929</v>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0501.png</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr"/>
+      <c r="D931" t="inlineStr"/>
+      <c r="E931" t="inlineStr"/>
+      <c r="F931" t="inlineStr">
+        <is>
+          <t>COc1ccc(CC(=O)N2CC[C@@H](Oc3ccc(-c4cn(CCCC(=O)NCCCCCCCNc5cccc6c5C(=O)N(C5CCC(=O)NC5=O)C6=O)cn4)cc3C(N)=O)[C@H](F)C2)cc1</t>
+        </is>
+      </c>
+      <c r="G931" t="inlineStr"/>
+      <c r="H931" t="inlineStr"/>
+      <c r="I931" t="n">
+        <v>0.8179582863868883</v>
+      </c>
+      <c r="J931" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K931" t="inlineStr"/>
+    </row>
+    <row r="932">
+      <c r="A932" s="1" t="n">
+        <v>930</v>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0509.png</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr"/>
+      <c r="D932" t="inlineStr"/>
+      <c r="E932" t="inlineStr"/>
+      <c r="F932" t="inlineStr">
+        <is>
+          <t>[H]c1c2cc(C(=O)N(C(C)C)C(C)C)cc1-n1nnc(c1[H])-c1cc(C(=O)N(C(C)C)C(C)C)cc(c1[H])-n1nnc(c1[H])-c1cc(C(=O)N(C(C)C)C(C)C)cc(c1[H])-n1nnc(c1[H])-c1cc(C(=O)N(C(C)C)C(C)C)cc(c1[H])-n1nnc-2c1[H]</t>
+        </is>
+      </c>
+      <c r="G932" t="inlineStr"/>
+      <c r="H932" t="inlineStr"/>
+      <c r="I932" t="n">
+        <v>0.5856722169946543</v>
+      </c>
+      <c r="J932" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K932" t="inlineStr"/>
+    </row>
+    <row r="933">
+      <c r="A933" s="1" t="n">
+        <v>931</v>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0510.png</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr"/>
+      <c r="D933" t="inlineStr"/>
+      <c r="E933" t="inlineStr"/>
+      <c r="F933" t="inlineStr">
+        <is>
+          <t>O=C(O)C1=CC234=C(C=C1)N=C1(CC5678=CC=C9%10C%11=CC9%12%13=NC(=CC=C%12)OCC9=C(C=C(C%12=CN(C%14CC%14)N=C%12)C=C9)CCCCOC59=C%10C%11%13=CC=6=C97C8C5=N1C=2=CN53CC1CCO1)N4CC1CCO1</t>
+        </is>
+      </c>
+      <c r="G933" t="inlineStr"/>
+      <c r="H933" t="inlineStr"/>
+      <c r="I933" t="n">
+        <v>0.008656474772805357</v>
+      </c>
+      <c r="J933" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K933" t="inlineStr"/>
+    </row>
+    <row r="934">
+      <c r="A934" s="1" t="n">
+        <v>932</v>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0517.png</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr"/>
+      <c r="D934" t="inlineStr"/>
+      <c r="E934" t="inlineStr"/>
+      <c r="F934" t="inlineStr">
+        <is>
+          <t>CC(C)C(NC(=O)CCOCCOCCOCCOCCC(=O)N1CCN(C(=O)C2=CC(F)=C(NC34=NC(C5CC5)=C5N678C9%10=C%11=C6%12%13(=CN6=C37N59%12C=648=N%11)C3(=CNN=C3)C3=NNC=C3%10%13)C=C2)CC1)C(=O)N1CC(O)CC1C(=O)NCC1=CC=C(C2=CN=CS2)C=C1</t>
+        </is>
+      </c>
+      <c r="G934" t="inlineStr"/>
+      <c r="H934" t="inlineStr"/>
+      <c r="I934" t="n">
+        <v>0.02367715968557669</v>
+      </c>
+      <c r="J934" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K934" t="inlineStr"/>
+    </row>
+    <row r="935">
+      <c r="A935" s="1" t="n">
+        <v>933</v>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0520.png</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr"/>
+      <c r="D935" t="inlineStr"/>
+      <c r="E935" t="inlineStr"/>
+      <c r="F935" t="inlineStr">
+        <is>
+          <t>CCN12C(C3=C(C(C)OC)N=CC(N4CCN(C)CC4)=C3)=C34=C1(C1=C(C(C)OC)N=CC(N5CCN(C)CC5)=C1)=C1CC(C)(C)COC(=O)[CH]NN5(CC6(C)C(C(N5)C(=O)OCC(C)(C)C3)C6(F)F)C(=O)C(NC(=O)C3CC3C)CC3=NC(=CS3)C35=CC=C2(C1=C3)C4=C5</t>
+        </is>
+      </c>
+      <c r="G935" t="inlineStr"/>
+      <c r="H935" t="inlineStr"/>
+      <c r="I935" t="n">
+        <v>0.3934247189193844</v>
+      </c>
+      <c r="J935" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K935" t="inlineStr"/>
+    </row>
+    <row r="936">
+      <c r="A936" s="1" t="n">
+        <v>934</v>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0522.png</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr"/>
+      <c r="D936" t="inlineStr"/>
+      <c r="E936" t="inlineStr"/>
+      <c r="F936" t="inlineStr">
+        <is>
+          <t>[H][C@]12CC(C)(C)[C@@H](C(=O)N[C@H](CCC(=O)NCCNC(=O)CC[C@@H](NC(=O)[C@H]3N4C(=O)[C@@H](NC(=O)[C@H](C)N(C)C(=O)OC(C)(C)C)CCS[C@@]4([H])CC3(C)C)c3ccccc3)c3ccccc3)N1C(=O)[C@@H](NC(=O)[C@H](C)N(C)C(=O)OC(C)(C)C)CCS2</t>
+        </is>
+      </c>
+      <c r="G936" t="inlineStr"/>
+      <c r="H936" t="inlineStr"/>
+      <c r="I936" t="n">
+        <v>0.7626757112394875</v>
+      </c>
+      <c r="J936" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K936" t="inlineStr"/>
+    </row>
+    <row r="937">
+      <c r="A937" s="1" t="n">
+        <v>935</v>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0524.png</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr"/>
+      <c r="D937" t="inlineStr"/>
+      <c r="E937" t="inlineStr"/>
+      <c r="F937" t="inlineStr">
+        <is>
+          <t>COC(=O)COC1=C(N2CCOCCOCCN(C3=CC4=C(C=C3O3CC3(=O)OC)C3(OC4=O)C4=C(C=C(OC(C)=O)C(C5=CC=NC=C5)=C4)OC4=C3C=C(C3=CC=NC=C3)C(OC(C)=O)=C4)CCOCC2)C=CC=C1</t>
+        </is>
+      </c>
+      <c r="G937" t="inlineStr"/>
+      <c r="H937" t="inlineStr"/>
+      <c r="I937" t="n">
+        <v>0.3529091629746254</v>
+      </c>
+      <c r="J937" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K937" t="inlineStr"/>
+    </row>
+    <row r="938">
+      <c r="A938" s="1" t="n">
+        <v>936</v>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0526.png</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr"/>
+      <c r="D938" t="inlineStr"/>
+      <c r="E938" t="inlineStr"/>
+      <c r="F938" t="inlineStr">
+        <is>
+          <t>C=C1=C2(C(=O)N3CCN(CC(=O)NCCOCCOCCOCC(=O)NC(C(=O)N4CC(O)CC4C(=O)NCC4=CC=C(C5=C(C)N=CS5)C=C4)C(C)(C)C)CC3)=CC(F)=C34NC56789=NC%10=CN%11%12C%13%14%15%16=CN=C%115%17%18C65(=N=7C6(=C7N%13%17%11%19C%13%17(=CN=C%125%118N7%13%14%18%19)C%155=CNN=C5C%17%165=CNN=C5)C5CC5C%1065CC5)N39C(=C1F)C4=C2</t>
+        </is>
+      </c>
+      <c r="G938" t="inlineStr"/>
+      <c r="H938" t="inlineStr"/>
+      <c r="I938" t="n">
+        <v>0.003147282892074059</v>
+      </c>
+      <c r="J938" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K938" t="inlineStr"/>
+    </row>
+    <row r="939">
+      <c r="A939" s="1" t="n">
+        <v>937</v>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0529.png</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr"/>
+      <c r="D939" t="inlineStr"/>
+      <c r="E939" t="inlineStr"/>
+      <c r="F939" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC1=NC2=C3N1CC=CCN145C67=C89C%10=C(C(N)=O)C=C6%11OCC6%12%13COC3(=CC(C(N)=O)=C2)OCC(C6OC72=CC(C(N)=O)=C8C%1036=C%1121NC41(NC(=O)C2=CC(C)=NN2CC)(=N3)=N96=C51NC(=O)C1=CC(C)=NN1CC)C%12C1(CN(C)C1)C%13</t>
+        </is>
+      </c>
+      <c r="G939" t="inlineStr"/>
+      <c r="H939" t="inlineStr"/>
+      <c r="I939" t="n">
+        <v>0.01641490567281529</v>
+      </c>
+      <c r="J939" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K939" t="inlineStr"/>
+    </row>
+    <row r="940">
+      <c r="A940" s="1" t="n">
+        <v>938</v>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0530.png</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr"/>
+      <c r="D940" t="inlineStr"/>
+      <c r="E940" t="inlineStr"/>
+      <c r="F940" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC1=NC2=C3C(=CC(C(N)=O)=C2)OCC(N2CCC(C(=O)O)CC2)COC24=CC(C(N)=O)=CC567=C2(C(OCC(CO)N2CCC(C(=O)O)CC2)=C=4C(C(N)=O)=C5)N2(CC=CCN13)C(NC(=O)C1=CC(C)=NN1CC)=N6C2(NC(=O)C1=CC(C)=NN1CC)=N7</t>
+        </is>
+      </c>
+      <c r="G940" t="inlineStr"/>
+      <c r="H940" t="inlineStr"/>
+      <c r="I940" t="n">
+        <v>0.1373248101091842</v>
+      </c>
+      <c r="J940" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K940" t="inlineStr"/>
+    </row>
+    <row r="941">
+      <c r="A941" s="1" t="n">
+        <v>939</v>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0532.png</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr"/>
+      <c r="D941" t="inlineStr"/>
+      <c r="E941" t="inlineStr"/>
+      <c r="F941" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC1=N2C3(NC(=O)C4=CC(C)=NN4CC)=NC245=C2(C=CC(C(N)=O)=C4)C(=CC(C(N)=O)=C5)OCC(N4CCC(C(=O)O)C4)COC4=CC(C(N)=O)=CC=C4NCC=CCN132</t>
+        </is>
+      </c>
+      <c r="G941" t="inlineStr"/>
+      <c r="H941" t="inlineStr"/>
+      <c r="I941" t="n">
+        <v>0.49137262394176</v>
+      </c>
+      <c r="J941" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K941" t="inlineStr"/>
+    </row>
+    <row r="942">
+      <c r="A942" s="1" t="n">
+        <v>940</v>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0533.png</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr"/>
+      <c r="D942" t="inlineStr"/>
+      <c r="E942" t="inlineStr"/>
+      <c r="F942" t="inlineStr">
+        <is>
+          <t>COC1C=COC(C)OC2=C3(C)C(O)=CC45(=O)C67=C(O)C(C)=C238OC2(C)OC=CC(OC)[CH]1(C)C(OC(C)=O)C(C)C(O)C(C)C(O)C(C)C=CC=C(C)C(=O)N1C43=C49O%10C%11%12=C(N=C4(C6=C8C2=O)C%103(=C195C7=O)O%11)C(O)=CC(OCCNC(C)=O)=C%12</t>
+        </is>
+      </c>
+      <c r="G942" t="inlineStr"/>
+      <c r="H942" t="inlineStr"/>
+      <c r="I942" t="n">
+        <v>0.01162381732013528</v>
+      </c>
+      <c r="J942" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K942" t="inlineStr"/>
+    </row>
+    <row r="943">
+      <c r="A943" s="1" t="n">
+        <v>941</v>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0535.png</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr"/>
+      <c r="D943" t="inlineStr"/>
+      <c r="E943" t="inlineStr"/>
+      <c r="F943" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC12=NC34=C56=C7C=C(C(N)=O)C=C58OCC5CO9C%10OC9%11=CC(C(N)=O)=CC9%12=C%11%13N%11CC=CCN1C=38(C(=CC(C(N)=O)=C74)OCC%10(C1=CC=CC=N1)C51=CC=CC=N1)N26CC=CCN%13C1(=N9)=N%12=C%11NC(=O)C2=CC(C)=NN2(CC)C2(=CC(C)=NN2CC)C(=O)N1</t>
+        </is>
+      </c>
+      <c r="G943" t="inlineStr"/>
+      <c r="H943" t="inlineStr"/>
+      <c r="I943" t="n">
+        <v>0.002630635169755023</v>
+      </c>
+      <c r="J943" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K943" t="inlineStr"/>
+    </row>
+    <row r="944">
+      <c r="A944" s="1" t="n">
+        <v>942</v>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0536.png</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr"/>
+      <c r="D944" t="inlineStr"/>
+      <c r="E944" t="inlineStr"/>
+      <c r="F944" t="inlineStr">
+        <is>
+          <t>CC1=C(C2=CC=C(CNC(=O)C3CC(O)CN3C(=O)C(NC(=O)COCCOCCOCCNC(=O)CN3CCN(C(=O)C4=CC(F)=C(NC56=NC(C7CC7)=C7N89%10C%11%12=C%13=C8%14%15(=CN8=C59%16N7%11%14C=86%16%10=N%13)C%125=C6=C%157(=CNN=C7)C5=NN6)C=C4)CC3)C(C)(C)C)C=C2)C=CN1</t>
+        </is>
+      </c>
+      <c r="G944" t="inlineStr"/>
+      <c r="H944" t="inlineStr"/>
+      <c r="I944" t="n">
+        <v>0.01114003974878576</v>
+      </c>
+      <c r="J944" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K944" t="inlineStr"/>
+    </row>
+    <row r="945">
+      <c r="A945" s="1" t="n">
+        <v>943</v>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0538.png</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr"/>
+      <c r="D945" t="inlineStr"/>
+      <c r="E945" t="inlineStr"/>
+      <c r="F945" t="inlineStr">
+        <is>
+          <t>Cc1ncsc1-c1ccc(CNC(=O)[C@@H]2C[C@@H](O)CN2C(=O)[C@@H](NC(=O)CCOCCC(=O)NCCCCn2cnc(-c3cnc(O[C@@H]4CCN(C(=O)Cc5ccc(OC(F)(F)F)cc5)C[C@H]4F)c(C(N)=O)c3)c2)C(C)(C)C)cc1</t>
+        </is>
+      </c>
+      <c r="G945" t="inlineStr"/>
+      <c r="H945" t="inlineStr"/>
+      <c r="I945" t="n">
+        <v>0.8399942643559993</v>
+      </c>
+      <c r="J945" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K945" t="inlineStr"/>
+    </row>
+    <row r="946">
+      <c r="A946" s="1" t="n">
+        <v>944</v>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0539.png</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr"/>
+      <c r="D946" t="inlineStr"/>
+      <c r="E946" t="inlineStr"/>
+      <c r="F946" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC1=NC2=C3C(=CC(C(=O)O)=C2)OCC2(N4CCC(O[Si](C)(C)C(C)(C)C)C4)COC45=CC(C(=O)O)=CC678=C4(C(=C=5C(C(=O)O)=C6)OC2CN2CCC(O[Si](C)(C)C(C)(C)C)C2)N(CC=CCN13)(C(NC(=O)C1=CC(C)=NN1CC)=N7)C(NC(=O)C1=CC(C)=NN1CC)=N8</t>
+        </is>
+      </c>
+      <c r="G946" t="inlineStr"/>
+      <c r="H946" t="inlineStr"/>
+      <c r="I946" t="n">
+        <v>0.09876894263902443</v>
+      </c>
+      <c r="J946" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K946" t="inlineStr"/>
+    </row>
+    <row r="947">
+      <c r="A947" s="1" t="n">
+        <v>945</v>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0540.png</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr"/>
+      <c r="D947" t="inlineStr"/>
+      <c r="E947" t="inlineStr"/>
+      <c r="F947" t="inlineStr">
+        <is>
+          <t>NC(=O)c1cc(-c2cn(CCCCNC(=O)CCOCCOCCNc3cccc4c3C(=O)N(C3CCC(=O)NC3=O)C4=O)cn2)cnc1O[C@@H]1CCN(C(=O)Cc2ccc(OC(F)(F)F)cc2)C[C@H]1F</t>
+        </is>
+      </c>
+      <c r="G947" t="inlineStr"/>
+      <c r="H947" t="inlineStr"/>
+      <c r="I947" t="n">
+        <v>0.8400529315157256</v>
+      </c>
+      <c r="J947" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K947" t="inlineStr"/>
+    </row>
+    <row r="948">
+      <c r="A948" s="1" t="n">
+        <v>946</v>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0541.png</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr"/>
+      <c r="D948" t="inlineStr"/>
+      <c r="E948" t="inlineStr"/>
+      <c r="F948" t="inlineStr">
+        <is>
+          <t>[H]C12CC3(CC=CC3)C(C(=O)NC3C4=C(C=CC=C4)CC3OCC#CC#CCO[CH]3=CC4=C(C=CC=C4)C3NC(=O)C3N4C(=O)C(NC(=O)C(C)NC)CCSC4([H])CC34CC=CC4)N1C(=O)C(NC(=O)C(C)NC)CCS2</t>
+        </is>
+      </c>
+      <c r="G948" t="inlineStr"/>
+      <c r="H948" t="inlineStr"/>
+      <c r="I948" t="n">
+        <v>0.6619135757376027</v>
+      </c>
+      <c r="J948" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K948" t="inlineStr"/>
+    </row>
+    <row r="949">
+      <c r="A949" s="1" t="n">
+        <v>947</v>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0546.png</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr"/>
+      <c r="D949" t="inlineStr"/>
+      <c r="E949" t="inlineStr"/>
+      <c r="F949" t="inlineStr">
+        <is>
+          <t>C1C2[C-]3C2O13.[C-]#[N+]C1=C2C3=C4C=C1C1([N+]#[C-])=CC25=C2(C=C1)COC167=CC=C8(F)C9(=N1)C1(F)=CC=C(N6=C18C9(=CC=CCC1=NC6=C(C=C([C-]=O)C=C6OCCOC)N1CC1CCO1)C=CCOCC35)O7C42</t>
+        </is>
+      </c>
+      <c r="G949" t="inlineStr"/>
+      <c r="H949" t="inlineStr"/>
+      <c r="I949" t="n">
+        <v>0.01955401887429398</v>
+      </c>
+      <c r="J949" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K949" t="inlineStr"/>
+    </row>
+    <row r="950">
+      <c r="A950" s="1" t="n">
+        <v>948</v>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0556.png</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr"/>
+      <c r="D950" t="inlineStr"/>
+      <c r="E950" t="inlineStr"/>
+      <c r="F950" t="inlineStr">
+        <is>
+          <t>COc1cc(-c2cn(C)c(=O)c3cc(C(=O)NCC4CC5(CCN(CCN6CCN(c7ccc8c(c7)C(=O)N(C7CCC(=O)NC7=O)C8=O)CC6)CC5)CO4)sc23)cc(OC)c1CN(C)C</t>
+        </is>
+      </c>
+      <c r="G950" t="inlineStr"/>
+      <c r="H950" t="inlineStr"/>
+      <c r="I950" t="n">
+        <v>0.8246892665782795</v>
+      </c>
+      <c r="J950" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K950" t="inlineStr"/>
+    </row>
+    <row r="951">
+      <c r="A951" s="1" t="n">
+        <v>949</v>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0557.png</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr"/>
+      <c r="D951" t="inlineStr"/>
+      <c r="E951" t="inlineStr"/>
+      <c r="F951" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC1=NC2=C3C(=CC(C(N)=O)=C2)OCC2(CCC4CCOCN4)COC456=CC(C(N)=O)=CC789=C4(C(=C=5C(C(N)=O)=C7)O6C2)N2(CC=CCN13)C(NC(=O)C1=CC(C)=NN1CC)=N8C2(NC(=O)C1=CC(C)=NN1CC)=N9</t>
+        </is>
+      </c>
+      <c r="G951" t="inlineStr"/>
+      <c r="H951" t="inlineStr"/>
+      <c r="I951" t="n">
+        <v>0.2430776260328035</v>
+      </c>
+      <c r="J951" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K951" t="inlineStr"/>
+    </row>
+    <row r="952">
+      <c r="A952" s="1" t="n">
+        <v>950</v>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0564.png</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr"/>
+      <c r="D952" t="inlineStr"/>
+      <c r="E952" t="inlineStr"/>
+      <c r="F952" t="inlineStr">
+        <is>
+          <t>C=C(C=CC=CC=CC1=CC=CC=C1)C1=C2(C=CC=C1)[C]13(=CC456=[C]789C%10%11%12=C1C%1071%13=[C]%117%10C%11=CC=CC7%14=[C]%111[Pt]38%1017%11%15%16%17[N]3=C(C=CC=C3)C3=[C]1(C=CC(=C)=C1=CC=C[C]47(=C1C1=C[C]%114=C(C=C1)C1=[N]4%15C=CC=C1)=[C]59%16=[C]%126%13%17)C=C%14C=C3)C213=N2C=CC=CC2=C1C=CC=C3</t>
+        </is>
+      </c>
+      <c r="G952" t="inlineStr"/>
+      <c r="H952" t="inlineStr"/>
+      <c r="I952" t="n">
+        <v>0.0006956235549215273</v>
+      </c>
+      <c r="J952" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K952" t="inlineStr"/>
+    </row>
+    <row r="953">
+      <c r="A953" s="1" t="n">
+        <v>951</v>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0566.png</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr"/>
+      <c r="D953" t="inlineStr"/>
+      <c r="E953" t="inlineStr"/>
+      <c r="F953" t="inlineStr">
+        <is>
+          <t>[C-]1CCO1.[C-]C(F)(F)CNCCOC1=CC(C(=O)O)=CC2=C1N=C(CC=CC=C13C4=C5C6(=CC=C4)O47C8C9=CC=C([N+]#[C-])C%10(=C9)C9([N+]#[C-])=C%11C=C8%12C=C9C%108([N+]#[C-])=CC%11=C9(C=C8)COC48%10%11=CC=C4C1%13%14=N8C431=N6%13%10C57(=CC=C%141)O%11C%129)N2CC1CCO1</t>
+        </is>
+      </c>
+      <c r="G953" t="inlineStr"/>
+      <c r="H953" t="inlineStr"/>
+      <c r="I953" t="n">
+        <v>0.002256801484788682</v>
+      </c>
+      <c r="J953" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K953" t="inlineStr"/>
+    </row>
+    <row r="954">
+      <c r="A954" s="1" t="n">
+        <v>952</v>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0570.png</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr"/>
+      <c r="D954" t="inlineStr"/>
+      <c r="E954" t="inlineStr"/>
+      <c r="F954" t="inlineStr">
+        <is>
+          <t>[H]C12CC(C)(C)C(C(=O)NC3C4=CC=CCC4=CC3OCC#CC#CCO[CH]3=CC4=C(C=CC=C4)C3NC(=O)C3N4C(=O)C(NC(=O)C(C)(C)NC)CCSC4([H])CC3(C)C)N1C(=O)C(NC(=O)C(C)(C)NC)CCS2</t>
+        </is>
+      </c>
+      <c r="G954" t="inlineStr"/>
+      <c r="H954" t="inlineStr"/>
+      <c r="I954" t="n">
+        <v>0.5544399125273991</v>
+      </c>
+      <c r="J954" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K954" t="inlineStr"/>
+    </row>
+    <row r="955">
+      <c r="A955" s="1" t="n">
+        <v>953</v>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0573.png</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr"/>
+      <c r="D955" t="inlineStr"/>
+      <c r="E955" t="inlineStr"/>
+      <c r="F955" t="inlineStr">
+        <is>
+          <t>[H]C12CC(C)(CC=C)C(C(=O)NC3C4=C(C=CC=C4)C=[CH]3OCC#CC#CCOC3C=C4CC=C=C=C4C3NC(=O)C3N4C(=O)C(NC(=O)C(C)NC)CCSC4([H])CC3(CC=C)CC=C)N1C(=O)C(NC(=O)C(C)NC)CCS2</t>
+        </is>
+      </c>
+      <c r="G955" t="inlineStr"/>
+      <c r="H955" t="inlineStr"/>
+      <c r="I955" t="n">
+        <v>0.251807944391749</v>
+      </c>
+      <c r="J955" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K955" t="inlineStr"/>
+    </row>
+    <row r="956">
+      <c r="A956" s="1" t="n">
+        <v>954</v>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0577.png</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr"/>
+      <c r="D956" t="inlineStr"/>
+      <c r="E956" t="inlineStr"/>
+      <c r="F956" t="inlineStr">
+        <is>
+          <t>Cl.[H]C12CCC(C(=O)NC3C4=C(C=CC=C4)C=[CH]3OCC#CC#CCOC3C=C4CC=CC=C4C3NC(=O)C3C(O)CC4([H])SCCC(NC(=O)C(C)NC)C(=O)N34)N1C(=O)C(NC(=O)C(C)NC)CCS2</t>
+        </is>
+      </c>
+      <c r="G956" t="inlineStr"/>
+      <c r="H956" t="inlineStr"/>
+      <c r="I956" t="n">
+        <v>0.4977714984601495</v>
+      </c>
+      <c r="J956" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K956" t="inlineStr"/>
+    </row>
+    <row r="957">
+      <c r="A957" s="1" t="n">
+        <v>955</v>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0579.png</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr"/>
+      <c r="D957" t="inlineStr"/>
+      <c r="E957" t="inlineStr"/>
+      <c r="F957" t="inlineStr">
+        <is>
+          <t>COc1cc(-c2cn(C)c(=O)c3cc(C(=O)NC4CCN(C5CCN(c6ccc7c(c6)CN(C6CCC(=O)NC6=O)C7=O)CC5(F)F)CC4)sc23)cc(OC)c1CN(C)C</t>
+        </is>
+      </c>
+      <c r="G957" t="inlineStr"/>
+      <c r="H957" t="inlineStr"/>
+      <c r="I957" t="n">
+        <v>0.7189004129747113</v>
+      </c>
+      <c r="J957" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K957" t="inlineStr"/>
+    </row>
+    <row r="958">
+      <c r="A958" s="1" t="n">
+        <v>956</v>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0580.png</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr"/>
+      <c r="D958" t="inlineStr"/>
+      <c r="E958" t="inlineStr"/>
+      <c r="F958" t="inlineStr">
+        <is>
+          <t>[H]C1([N+]#[C-])CC(F)(F)CN12C(=O)CNC(C)(=O)C1(=CC=NC3=CC=C(OCCCN4CCN(C(=O)C(CCCCNC(=O)CN5CCN(CC(=O)O)CCN(CC(=O)O)CCN(CC(=O)O)CC5)NC(=O)CCCC(=O)NC(CCCCNC(=O)CCCC5=CC=C(I)C=C5)C(=O)O)CC4)C=C31)C(=O)NCC(=O)N1CC(F)(F)CC12([H])[N+]#[C-]</t>
+        </is>
+      </c>
+      <c r="G958" t="inlineStr"/>
+      <c r="H958" t="inlineStr"/>
+      <c r="I958" t="n">
+        <v>0.509621557110935</v>
+      </c>
+      <c r="J958" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K958" t="inlineStr"/>
+    </row>
+    <row r="959">
+      <c r="A959" s="1" t="n">
+        <v>957</v>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0581.png</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr"/>
+      <c r="D959" t="inlineStr"/>
+      <c r="E959" t="inlineStr"/>
+      <c r="F959" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC=NC1=C23C4=CC(C(N)=O)=C1C1=C5N2CC=CCN26C7=CC8=C(C(N)=O)C=C7(OCC(C7CNC7)CO4)C24=C8(C=C(C(N)=O)C=C4OCC(C2CNC2)COC53=CC(C(N)=O)=C1)N=C6NC(=O)C1=CC(C)=NN1CC</t>
+        </is>
+      </c>
+      <c r="G959" t="inlineStr"/>
+      <c r="H959" t="inlineStr"/>
+      <c r="I959" t="n">
+        <v>0.1603132355197553</v>
+      </c>
+      <c r="J959" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K959" t="inlineStr"/>
+    </row>
+    <row r="960">
+      <c r="A960" s="1" t="n">
+        <v>958</v>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0582.png</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr"/>
+      <c r="D960" t="inlineStr"/>
+      <c r="E960" t="inlineStr"/>
+      <c r="F960" t="inlineStr">
+        <is>
+          <t>CC1=NOC(C(C(=O)N2CC(O)CC2C(=O)NC(CC(=O)NCCOCCOCCOCCNC(=O)CN23CCN4C5(=O)N(CC2)(CC3)C42(=O)C3=C4=C5267=CC(F)=C(C=C6)NC2568=NC9%10(C%11CC%11)=C%11N%12%13C%14=C(C9%15CC%15)N=%102=C2(N5C(=C4F)C=C=73)C634=NC2%1285=N=3C=C%13(C2=CNN=C2)N%14%1145)C2=CC=C(C3=C(C)N=CS3)C=C2)C(C)C)=C1</t>
+        </is>
+      </c>
+      <c r="G960" t="inlineStr"/>
+      <c r="H960" t="inlineStr"/>
+      <c r="I960" t="n">
+        <v>0.001474417749027076</v>
+      </c>
+      <c r="J960" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K960" t="inlineStr"/>
+    </row>
+    <row r="961">
+      <c r="A961" s="1" t="n">
+        <v>959</v>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0585.png</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr"/>
+      <c r="D961" t="inlineStr"/>
+      <c r="E961" t="inlineStr"/>
+      <c r="F961" t="inlineStr">
+        <is>
+          <t>O.[H][C@]1(C)C/C(C)=C/[C@@]([H])(CC=C)C(=O)C[C@]([H])(O)[C@@]([H])(C)[C@@]([H])(C(C)=C[C@]2([H])CC[C@@]([H])(O)[C@]([H])(OC)C2)OC(=O)[C@]2([H])CCCCN2C(=O)C(=O)[C@]2(O)O[C@]([H])([C@@]([H])(OC)C1)[C@@]([H])(OC)C[C@@]2([H])C</t>
+        </is>
+      </c>
+      <c r="G961" t="inlineStr"/>
+      <c r="H961" t="inlineStr"/>
+      <c r="I961" t="n">
+        <v>0.5265892542131855</v>
+      </c>
+      <c r="J961" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K961" t="inlineStr"/>
+    </row>
+    <row r="962">
+      <c r="A962" s="1" t="n">
+        <v>960</v>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0586.png</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr"/>
+      <c r="D962" t="inlineStr"/>
+      <c r="E962" t="inlineStr"/>
+      <c r="F962" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC12=NC34=C56=C7C=C(C(N)=O)C=C58OCC5N9(CCNCC9)C9(COC%10=CC(C(N)=O)=CC%11%12=C%10%13N%10CC=CCN16C=38(C(=CC(C(N)=O)=C74)OC9)N2CC=CCN%131C2=N%11=C%101(=N%12)NC(=O)C1(=CC(C)=NN1CC)N1(CC)N=C(C)C=C1C(=O)N2)N51CCNCC1</t>
+        </is>
+      </c>
+      <c r="G962" t="inlineStr"/>
+      <c r="H962" t="inlineStr"/>
+      <c r="I962" t="n">
+        <v>0.02162091186534806</v>
+      </c>
+      <c r="J962" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K962" t="inlineStr"/>
+    </row>
+    <row r="963">
+      <c r="A963" s="1" t="n">
+        <v>961</v>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0588.png</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr"/>
+      <c r="D963" t="inlineStr"/>
+      <c r="E963" t="inlineStr"/>
+      <c r="F963" t="inlineStr">
+        <is>
+          <t>C1C2[C-]3C2O13.[C-]OC(=O)C1=CC2=C(N=C(CC=CC=C34C56=N789C%10%11=CC=C5%12C375=N%103C87%10(=CC=C65(F)C4%1239=N7)OCC34=C5C=C([N+]#[C-])(C=C3)C3=CC(=CC5=C3[N+]#[C-])C4O%11%10)N2CC2CCO2)C(OCCOC)=C1</t>
+        </is>
+      </c>
+      <c r="G963" t="inlineStr"/>
+      <c r="H963" t="inlineStr"/>
+      <c r="I963" t="n">
+        <v>0.03307572973154837</v>
+      </c>
+      <c r="J963" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K963" t="inlineStr"/>
+    </row>
+    <row r="964">
+      <c r="A964" s="1" t="n">
+        <v>962</v>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0591.png</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr"/>
+      <c r="D964" t="inlineStr"/>
+      <c r="E964" t="inlineStr"/>
+      <c r="F964" t="inlineStr">
+        <is>
+          <t>CCN1N=C(C)C=C1C(=O)NC1=NC2=C3C(=CC(C(=O)OC)=C2)OCC24(N5CCC(O[Si](C)(C)C(C)(C)C)C5)COC56=CC(C(=O)OC)=CC789=C5(C(=C=6C(C(=O)OC)=C7)OC2C(N2CCC(O[Si](C)(C)C(C)(C)C)C2)C4O)N(CC=CCN13)(C(NC(=O)C1=CC(C)=NN1CC)=N8)C(NC(=O)C1=CC(C)=NN1CC)=N9</t>
+        </is>
+      </c>
+      <c r="G964" t="inlineStr"/>
+      <c r="H964" t="inlineStr"/>
+      <c r="I964" t="n">
+        <v>0.00662854049889302</v>
+      </c>
+      <c r="J964" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K964" t="inlineStr"/>
+    </row>
+    <row r="965">
+      <c r="A965" s="1" t="n">
+        <v>963</v>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0593.png</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr"/>
+      <c r="D965" t="inlineStr"/>
+      <c r="E965" t="inlineStr"/>
+      <c r="F965" t="inlineStr">
+        <is>
+          <t>CC1=C(C2=CC=C(CNC(=O)C3CC(O)CN3C(=O)C(NC(=O)CCCC(=O)NCCN3CCN(C(=O)C456=CC(F)=C78C(=C4)C(=C(F)C=5=C6)N74C567=N9=C45%10(=NC4=C5N%11C%12(C%13=CNN=C%13)=CN=C%116%10N5%12C=C9C5CC5C45CC5)N87)CC3)C(C)C)C=C2)SC=N1</t>
+        </is>
+      </c>
+      <c r="G965" t="inlineStr"/>
+      <c r="H965" t="inlineStr"/>
+      <c r="I965" t="n">
+        <v>0.05170676424581289</v>
+      </c>
+      <c r="J965" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K965" t="inlineStr"/>
+    </row>
+    <row r="966">
+      <c r="A966" s="1" t="n">
+        <v>964</v>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0594.png</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr"/>
+      <c r="D966" t="inlineStr"/>
+      <c r="E966" t="inlineStr"/>
+      <c r="F966" t="inlineStr">
+        <is>
+          <t>[H][C@]12CC3(CCCC3)[C@@H](C(=O)N[C@H]3c4ccccc4C[C@H]3OCC#CC#CCO[C@@H]3Cc4ccccc4[C@@H]3NC(=O)[C@H]3N4C(=O)[C@@H](NC(=O)[C@H](C)NC)CCO[C@@]4([H])CC34CCCC4)N1C(=O)[C@@H](NC(=O)[C@H](C)NC)CCO2</t>
+        </is>
+      </c>
+      <c r="G966" t="inlineStr"/>
+      <c r="H966" t="inlineStr"/>
+      <c r="I966" t="n">
+        <v>0.8249204783561979</v>
+      </c>
+      <c r="J966" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K966" t="inlineStr"/>
+    </row>
+    <row r="967">
+      <c r="A967" s="1" t="n">
+        <v>965</v>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0598.png</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr"/>
+      <c r="D967" t="inlineStr"/>
+      <c r="E967" t="inlineStr"/>
+      <c r="F967" t="inlineStr">
+        <is>
+          <t>COC1=CC(OCCN(C)C)=CC=C1N=C1C=C23NC(=O)C(C)=CC=CC(C)[CH]45(O)[CH](C)(C=CC=C(C)C(=O)N2)[CH]2(O)[CH]4(C)[CH]4(O)[CH]6(C)[CH](O)([CH]4(C)[CH]4(OC(C)=O)[CH]7(C)[CH]8(OC)C=CO9%10C(=CC(OC)[CH]84(C)[CH]67OC(C)=O)OC9467(C)OC89%11=C(C)C(O)=C(C3=O)C1=C8C4(=O)C%1096O%117)[CH]25C</t>
+        </is>
+      </c>
+      <c r="G967" t="inlineStr"/>
+      <c r="H967" t="inlineStr"/>
+      <c r="I967" t="n">
+        <v>0.002893464234439642</v>
+      </c>
+      <c r="J967" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K967" t="inlineStr"/>
+    </row>
+    <row r="968">
+      <c r="A968" s="1" t="n">
+        <v>966</v>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>/root/cmage-work/bigsa/cx_in_20261009T124239/rb_0599.png</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr"/>
+      <c r="D968" t="inlineStr"/>
+      <c r="E968" t="inlineStr"/>
+      <c r="F968" t="inlineStr">
+        <is>
+          <t>CC1=C(C2=CC=C(CNC(=O)C3CC(O)CN3C(=O)C(NC(=O)CCCCCCCCNC(=O)CN34CCN5C6(=O)N(CC3)(CC4)C53(=O)C4=C5=C6378=CC(F)=C(C=C7)NC3679=NC%10%11%12=CN%13%14%15%16C%17=CN=C3%13%18C3(=N=%106C(=C%14N%17%186C%15(C%10=CNN=C%10)=CN=C367%16)C%113CC3C%123CC3)N9C(=C5F)C=C=84)C(C)(C)C)C=C2)SC=N1</t>
+        </is>
+      </c>
+      <c r="G968" t="inlineStr"/>
+      <c r="H968" t="inlineStr"/>
+      <c r="I968" t="n">
+        <v>0.001199295675504335</v>
+      </c>
+      <c r="J968" t="inlineStr">
+        <is>
+          <t>Discard this SMILES prediction</t>
+        </is>
+      </c>
+      <c r="K968" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>